<commit_message>
Tercera version visual calendario
</commit_message>
<xml_diff>
--- a/calendario_iglesia_datos.xlsx
+++ b/calendario_iglesia_datos.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="1" r:id="R5ff2fdb293224362"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicios" sheetId="2" r:id="Re094bd2fa2cf4a33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados" sheetId="3" r:id="Rfe2add4206d24fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meses" sheetId="4" r:id="R890f81a78e0d4277"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro Servicios" sheetId="5" r:id="R8338c78a544d4a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="6" r:id="R9ab7a2e12cb54f21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidores" sheetId="1" r:id="R6da3d35450894aef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servicios" sheetId="2" r:id="R3dc9e9a7945641c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estados" sheetId="3" r:id="R63f7243222a44a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meses" sheetId="4" r:id="Ra7c9c05c45e24971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro Servicios" sheetId="5" r:id="R54f1f5f3c8714bc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuracion" sheetId="6" r:id="R32e458b9f1ac4d93"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,8 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="dd/mm/yyyy"/>
+    <x:numFmt numFmtId="203" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -33,12 +36,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="0F766E"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -53,7 +61,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -86,6 +94,26 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -463,7 +491,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2ff3a5e72f46e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84fc0369fa62446d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -557,7 +585,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cb5b4bc94504033"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reff9a4effed94302"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -597,7 +625,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R700574e647b34c14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11680feeff1744d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -717,7 +745,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2a4b0e1fccd4359"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf434ef7dd4df4bfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1474,7 +1502,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ceb3515b0d4d50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf161b2d1d2d04c51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1488,49 +1516,137 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="8" t="str">
+      <x:c r="A1" s="22" t="str">
         <x:v>Parametro</x:v>
       </x:c>
-      <x:c r="B1" s="8" t="str">
+      <x:c r="B1" s="22" t="str">
         <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C1" s="25" t="str">
+        <x:v>Descripción</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
+        <x:v>Editable</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="9" t="str">
         <x:v>CantidadGrupos</x:v>
       </x:c>
-      <x:c r="B2" s="9" t="n">
+      <x:c r="B2" s="17" t="n">
         <x:v>5</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Total de grupos de servicio.</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>Sí</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="9" t="str">
-        <x:v>FechaReferenciaSemana</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="n">
+        <x:v>FechaBaseRotacion</x:v>
+      </x:c>
+      <x:c r="B3" s="18" t="n">
         <x:v>46173</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Domingo de la semana conocida. Base fija para calcular la rotación.</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Sí</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
-        <x:v>GrupoReferencia</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="n">
+        <x:v>GrupoBaseRotacion</x:v>
+      </x:c>
+      <x:c r="B4" s="17" t="n">
         <x:v>5</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Grupo que sirvió en la semana base.</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Sí</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="9" t="str">
         <x:v>InicioSemana</x:v>
       </x:c>
-      <x:c r="B5" s="9" t="str">
+      <x:c r="B5" s="19" t="str">
         <x:v>Domingo</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>La app trabaja de domingo a sábado.</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>FechaSemanaActual</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="e">
+        <x:f>HOY()-DIASEM(HOY(),1)+1</x:f>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Domingo de la semana actual. En Excel se actualiza al abrir/recalcular.</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>GrupoActivoActual</x:v>
+      </x:c>
+      <x:c r="B7" s="21" t="e">
+        <x:f>RESIDUO(B3-1+ENTERO((B6-B2)/7),B1)+1</x:f>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Grupo que sirve esta semana según la rotación.</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>FechaReferenciaSemana</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="n">
+        <x:f>B2</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Compatibilidad: igual a FechaBaseRotacion.</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>GrupoReferencia</x:v>
+      </x:c>
+      <x:c r="B9" s="21" t="n">
+        <x:f>B3</x:f>
+        <x:v>46173</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Compatibilidad: igual a GrupoBaseRotacion.</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>No</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d21a9a144b40bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2b4ff0304024aa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>